<commit_message>
Expand literature matrix section placements
</commit_message>
<xml_diff>
--- a/outputs/literature_review_matrix.xlsx
+++ b/outputs/literature_review_matrix.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Lit Review Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Status Legend" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Source Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Section Integration" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Status Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Source Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lit Review Matrix'!$A$1:$F$57</definedName>
@@ -50,7 +51,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -72,11 +73,16 @@
         <color rgb="00D9E2F3"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +91,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -504,44 +516,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Claim / argument</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -883,7 +895,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Card game format</t>
+          <t>Literature review &gt; Card game format; System design &gt; Game condition</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -898,12 +910,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Among DCGs reviewed, only a small number relate to business/process contexts; use as example that card format is established but rare in sales/professional upskilling.</t>
+          <t>Use as card-format warrant and design caution: digital card games can support active learning, but scaffolding during play is still necessary.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mentioned; strengthen note</t>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1045,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; LM-GM extension</t>
+          <t>System design &gt; Design methodology; Literature review &gt; LM-GM lineage</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1048,7 +1060,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; could support design-development chapter, but not necessary unless supervisor wants deeper LM-GM lineage.</t>
+          <t>Candidate if the design-development chapter needs a stronger serious-game design-methodology lineage beyond Arnab et al. (2015).</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1063,7 +1075,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; DGBL design principles</t>
+          <t>Literature review &gt; DGBL design principles; System design &gt; Original design expectations</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1078,7 +1090,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; would strengthen the claim that the intervention hinges on pedagogical alignment.</t>
+          <t>Candidate if the thesis needs another design-review source for the claim that game elements must be connected to learning goals and mechanics.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1093,7 +1105,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Motivation mechanism</t>
+          <t>Literature review &gt; Gameful learning; Results and discussion &gt; H2 mechanism</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1108,12 +1120,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; useful if H2 motivational pathway needs stronger theory beyond Bandura.</t>
+          <t>Now integrated to support the claim that LM-GM alignment does not guarantee motivational meaning; mechanics must be interpreted through learner experience.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Potential add</t>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1315,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; CLT and games</t>
+          <t>Results and discussion &gt; Behavioral evidence; Future research &gt; Adaptive telemetry</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1318,12 +1330,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; strong candidate for telemetry/CL argument. Could support behavioral logs as CL-adjacent evidence.</t>
+          <t>Integrated in the telemetry/results section: supports theory-grounded log interpretation while warning that metrics can reflect stress, emotion, motor processes, or control familiarity, not only cognitive load.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Potential add</t>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1345,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; CLT and adult learners</t>
+          <t>Literature review &gt; Expertise reversal and learner readiness; Discussion &gt; cognitive-load interpretation</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1348,12 +1360,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; relevant to adult learner readiness and CL.</t>
+          <t>Integrated to support adult DGBL readiness: scaffolding effects depend on learner characteristics, so support is conditional rather than universally beneficial.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Potential add</t>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1675,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Telemetry</t>
+          <t>Limitations &gt; Behavioral telemetry; Results and discussion &gt; Behavioral evidence</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1678,7 +1690,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Important methodological caution for logs; already in limitations/discussion.</t>
+          <t>Use as methodological caution: trace data contextualize learning but do not capture the full self-regulatory process outside the platform.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1693,7 +1705,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Telemetry</t>
+          <t>Results and discussion &gt; Behavioral evidence; Limitations &gt; telemetry caution</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1708,7 +1720,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; could strengthen behavioral telemetry section, but may be non-game and general.</t>
+          <t>Candidate if a broader online-learning analytics citation is needed, but Sevcenko is more directly aligned with serious games and CL-adjacent telemetry.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1723,7 +1735,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Learning analytics in games</t>
+          <t>Future research &gt; Dynamic/adaptive telemetry; System design implications</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1738,7 +1750,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Supports future designs with telemetry-triggered routing/difficulty adjustment.</t>
+          <t>Supports learning analytics/game traces as design-improvement evidence and future telemetry-triggered adaptation.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1753,7 +1765,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Dynamic difficulty</t>
+          <t>Future research &gt; Dynamic difficulty adjustment</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1768,7 +1780,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Supports future implication and readiness-sensitive design.</t>
+          <t>Supports future readiness-sensitive adaptation and difficulty adjustment triggered by performance/latency thresholds.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1903,7 +1915,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Evaluation framework</t>
+          <t>Methodology &gt; Evaluation framing; Literature review &gt; DGBL evidence gap</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1918,7 +1930,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Unused duplicate items in Zotero; could support All et al. design/evaluation critique if one clean record is retained.</t>
+          <t>Candidate if the evaluation framework needs a broader educational-games lens beyond All et al.; keep one clean record only.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1963,7 +1975,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; DGBL meta-review</t>
+          <t>Literature review &gt; DGBL evidence base</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -1978,7 +1990,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Unused Zotero item; may be useful as a stronger general DGBL meta-analysis than some current broad claims.</t>
+          <t>Candidate for a broader DGBL meta-analytic anchor if current Wouters/Merchant/All framing needs reinforcement.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2023,7 +2035,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Gamification maturity</t>
+          <t>Literature review &gt; Gameful learning, mechanism, and learner context; Introduction &gt; contribution framing</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2038,12 +2050,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Useful mainly to avoid conflating gamification with game-based learning.</t>
+          <t>Integrated to justify the mature field-level question: how, when, and for whom gameful designs work.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Potential add</t>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2065,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Game enjoyment/performance</t>
+          <t>Results and discussion &gt; Engagement interpretation; Literature review &gt; engagement</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2068,7 +2080,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Could be used to discuss engagement, but less central than SE mediation.</t>
+          <t>Optional if engagement/enjoyment needs another empirical source; less central than self-efficacy mediation and Mekler.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2083,7 +2095,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Business training game precedent</t>
+          <t>Literature review &gt; Business/professional GBL precedent</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2098,7 +2110,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Potential example of business/professional GBL, but not sales-specific.</t>
+          <t>Optional business/process example; useful only if the sales/professional rarity claim needs another adjacent precedent.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2173,7 +2185,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Narrative contextual games</t>
+          <t>Results and discussion &gt; Within-game profile translation; Methodology &gt; exploratory analysis plan</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2188,7 +2200,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Important methodological model for clustering/profile table; already cited.</t>
+          <t>Primary methodological model for combining behavioral logs and psychometrics in the profile table; cited as adapted format, not name-dropped.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2203,7 +2215,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Literature review &gt; Practitioner sales card game</t>
+          <t>Literature review &gt; Practitioner sales card-game precedent; System design &gt; card format rationale</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2218,12 +2230,102 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Use carefully as non-peer-reviewed evidence of format precedent, not as theoretical support.</t>
+          <t>Non-peer-reviewed practitioner precedent only. Use carefully, if at all, to show format plausibility rather than theoretical support.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Potential add</t>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Literature review &gt; Gameful learning; Results and discussion &gt; H2 mechanism</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Game mechanics can alter observable behavior without producing the expected competence, autonomy, or intrinsic-motivation pathway.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Mekler et al. (2017)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Integrated to justify why engagement and telemetry are not treated as mechanisms by themselves; the thesis tests whether engagement travels through self-efficacy into ADAPTS-SV.</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>In manuscript</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Literature review &gt; Learner context; Discussion &gt; predictive readiness</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Expected value for gamified training depends on learner readiness toward the training technology, including game attitudes and prior game experience.</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Landers &amp; Armstrong (2017)</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Integrated as adjacent readiness evidence. Do not overclaim as sales-expertise moderation; use as support for the broader principle that gameful training is not uniformly received.</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>In manuscript</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Results and discussion &gt; Behavioral evidence; Cognitive Budget Framework operationalization</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Telemetry is useful for making friction visible, but it becomes psychological evidence only when interpreted with theory and psychometrics.</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Sevcenko et al. (2021); Lim et al. (2021); Mekler et al. (2017)</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Cross-section bridge: results use logs cautiously; discussion uses telemetry to operationalize mechanics acquisition cost; limitations protect against overclaim.</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>In manuscript</t>
         </is>
       </c>
     </row>
@@ -2259,113 +2361,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Suggested action</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="44" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>In manuscript</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Claim/reference is already represented in main.tex.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Keep unless prose is redundant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Mentioned; strengthen note</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Reference exists but could support a more precise claim.</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Add one sentence or footnote-level specificity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Potential add</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Useful source from Zotero or recent search, not yet integrated.</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Read/extract before adding; cite only if it strengthens the argument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Maybe omit</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Source is tangential, weakly aligned, duplicate, or lower quality.</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Do not add unless a specific gap appears.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Background only</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Useful for context/trend scanning, less useful for mechanism.</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Use sparingly, normally not central to argument.</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>References</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Use in thesis</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Manuscript action/status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Introduction / contribution framing</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>All et al. (2021); Nacke &amp; Deterding (2017)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Frame the study as relative effectiveness plus mechanism/for-whom evaluation, not a binary game-success claim.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Represented; keep concise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Literature review &gt; Sales education</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Cummins et al. (2013); Spiro &amp; Weitz (1990); Robinson et al. (2002); Cardinali et al. (2025)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Build sales education backbone and justify ADAPTS-SV as the applied adaptive-selling outcome.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Represented; ADAPTS-SV wording corrected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Literature review &gt; Gameful learning and mechanism</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Mekler et al. (2017); Landers &amp; Armstrong (2017); Proulx et al. (2017)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Demote engagement from explanation to tested mechanism; support readiness-sensitive reception of gameful training.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Represented in current manuscript.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Literature review &gt; CLT/readiness</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Kalyuga et al. (2003); Kalyuga (2007); Chang &amp; Yang (2023); Mayer (2009)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Anchor learner-relative load, expertise reversal, and mechanics as potentially costly processing.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Represented; supports Cognitive Budget Framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>System design and development</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Arnab et al. (2015); Kordaki &amp; Gousiou (2017); Mayer (2009)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Show the game was intentionally aligned through LM-GM/card mechanics while still carrying mechanics acquisition cost.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Represented; optional additions only if design-method lineage needs depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Methodology / analysis plan</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Chen et al. (2018); All et al. (2021)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Justify RCT + psychometrics + behavioral logs and the combined profile-table style.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Represented; avoid name-dropping by using citation language.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Results and discussion &gt; Behavioral evidence</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Sevcenko et al. (2021); Lim et al. (2021); Mekler et al. (2017)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Use telemetry as triangulation of gameplay friction and psychological pathways, not as a standalone cognitive-load or learning proxy.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Represented; Sevcenko is already in telemetry results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Results and discussion &gt; Within-game profiles</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Chen et al. (2018); Sevcenko et al. (2021)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Combine psychometrics and logs to translate clusters while keeping predictive and explanatory layers separate.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Discussion &gt; Cognitive Budget Framework</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Arnab et al. (2015); Plass et al. (2015); Kalyuga (2007); Sevcenko et al. (2021)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Operationalize mechanics acquisition cost, expertise offset, and effective load using design audit + pre-assessment + telemetry + CL measures.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Represented after latest branch cleanup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Future research</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Serrano-Laguna et al. (2012); Sevcenko et al. (2021); Zohaib (2018); Leppink et al. (2013)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Support telemetry-triggered adaptation, dynamic difficulty, and multidimensional cognitive-load measurement.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Represented.</t>
         </is>
       </c>
     </row>
@@ -2380,10 +2623,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>In manuscript</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Claim/reference is already represented in main.tex.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Keep unless prose is redundant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Mentioned; strengthen note</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Reference exists but could support a more precise claim.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Add one sentence or footnote-level specificity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Potential add</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Useful source from Zotero or recent search, not yet integrated.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Read/extract before adding; cite only if it strengthens the argument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Maybe omit</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Source is tangential, weakly aligned, duplicate, or lower quality.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Do not add unless a specific gap appears.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Useful for context/trend scanning, less useful for mechanism.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Use sparingly, normally not central to argument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Cross-section note</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>A reference may belong in Results, Discussion, Methodology, or Future Research even if first discovered during the literature-review audit.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Use the Location field and Section Integration sheet to avoid forcing every source into Chapter 2.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2447,6 +2828,30 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:43:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Update note</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Expanded potential-add tracking into cross-section placement, especially telemetry/results and future adaptive-design use.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>